<commit_message>
Sync project context and local data updates
</commit_message>
<xml_diff>
--- a/live_data/shop_sales_test_dataset_100_rows.xlsx
+++ b/live_data/shop_sales_test_dataset_100_rows.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
@@ -649,16 +649,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </bottom>
       <diagonal/>
     </border>
@@ -668,10 +668,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -969,7 +969,7 @@
   <dimension ref="A1:N101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1277,7 +1277,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1585,7 +1585,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1761,7 +1761,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1893,7 +1893,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27">
       <c r="A27" t="s">
         <v>39</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29">
       <c r="A29" t="s">
         <v>41</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32">
       <c r="A32" t="s">
         <v>44</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33">
       <c r="A33" t="s">
         <v>45</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34">
       <c r="A34" t="s">
         <v>46</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35">
       <c r="A35" t="s">
         <v>47</v>
       </c>
@@ -2509,7 +2509,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37">
       <c r="A37" t="s">
         <v>49</v>
       </c>
@@ -2597,7 +2597,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -2641,7 +2641,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39">
       <c r="A39" t="s">
         <v>51</v>
       </c>
@@ -2685,7 +2685,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40">
       <c r="A40" t="s">
         <v>52</v>
       </c>
@@ -2729,7 +2729,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41">
       <c r="A41" t="s">
         <v>53</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42">
       <c r="A42" t="s">
         <v>54</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43">
       <c r="A43" t="s">
         <v>55</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44">
       <c r="A44" t="s">
         <v>56</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45">
       <c r="A45" t="s">
         <v>57</v>
       </c>
@@ -2949,7 +2949,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46">
       <c r="A46" t="s">
         <v>58</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47">
       <c r="A47" t="s">
         <v>59</v>
       </c>
@@ -3037,7 +3037,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48">
       <c r="A48" t="s">
         <v>60</v>
       </c>
@@ -3081,7 +3081,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49">
       <c r="A49" t="s">
         <v>61</v>
       </c>
@@ -3125,7 +3125,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50">
       <c r="A50" t="s">
         <v>62</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51">
       <c r="A51" t="s">
         <v>63</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52">
       <c r="A52" t="s">
         <v>64</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53">
       <c r="A53" t="s">
         <v>65</v>
       </c>
@@ -3301,7 +3301,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54">
       <c r="A54" t="s">
         <v>66</v>
       </c>
@@ -3345,7 +3345,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55">
       <c r="A55" t="s">
         <v>67</v>
       </c>
@@ -3389,7 +3389,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -3433,7 +3433,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="57" spans="1:14">
+    <row r="57">
       <c r="A57" t="s">
         <v>69</v>
       </c>
@@ -3477,7 +3477,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58">
       <c r="A58" t="s">
         <v>70</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59">
       <c r="A59" t="s">
         <v>71</v>
       </c>
@@ -3565,7 +3565,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60">
       <c r="A60" t="s">
         <v>72</v>
       </c>
@@ -3609,7 +3609,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61">
       <c r="A61" t="s">
         <v>73</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="62" spans="1:14">
+    <row r="62">
       <c r="A62" t="s">
         <v>74</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="63" spans="1:14">
+    <row r="63">
       <c r="A63" t="s">
         <v>75</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64">
       <c r="A64" t="s">
         <v>76</v>
       </c>
@@ -3785,7 +3785,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65">
       <c r="A65" t="s">
         <v>77</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66">
       <c r="A66" t="s">
         <v>78</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67">
       <c r="A67" t="s">
         <v>79</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68">
       <c r="A68" t="s">
         <v>80</v>
       </c>
@@ -3961,7 +3961,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69">
       <c r="A69" t="s">
         <v>81</v>
       </c>
@@ -4005,7 +4005,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70">
       <c r="A70" t="s">
         <v>82</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71">
       <c r="A71" t="s">
         <v>83</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72">
       <c r="A72" t="s">
         <v>84</v>
       </c>
@@ -4137,7 +4137,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73">
       <c r="A73" t="s">
         <v>85</v>
       </c>
@@ -4181,7 +4181,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74">
       <c r="A74" t="s">
         <v>86</v>
       </c>
@@ -4225,7 +4225,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75">
       <c r="A75" t="s">
         <v>87</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76">
       <c r="A76" t="s">
         <v>88</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77">
       <c r="A77" t="s">
         <v>89</v>
       </c>
@@ -4357,7 +4357,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78">
       <c r="A78" t="s">
         <v>90</v>
       </c>
@@ -4401,7 +4401,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="79" spans="1:14">
+    <row r="79">
       <c r="A79" t="s">
         <v>91</v>
       </c>
@@ -4445,7 +4445,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="80" spans="1:14">
+    <row r="80">
       <c r="A80" t="s">
         <v>92</v>
       </c>
@@ -4489,7 +4489,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="81" spans="1:14">
+    <row r="81">
       <c r="A81" t="s">
         <v>93</v>
       </c>
@@ -4533,7 +4533,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="82" spans="1:14">
+    <row r="82">
       <c r="A82" t="s">
         <v>94</v>
       </c>
@@ -4577,7 +4577,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="83" spans="1:14">
+    <row r="83">
       <c r="A83" t="s">
         <v>95</v>
       </c>
@@ -4621,7 +4621,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="84" spans="1:14">
+    <row r="84">
       <c r="A84" t="s">
         <v>96</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="85" spans="1:14">
+    <row r="85">
       <c r="A85" t="s">
         <v>97</v>
       </c>
@@ -4709,7 +4709,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="86" spans="1:14">
+    <row r="86">
       <c r="A86" t="s">
         <v>98</v>
       </c>
@@ -4753,7 +4753,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="87" spans="1:14">
+    <row r="87">
       <c r="A87" t="s">
         <v>99</v>
       </c>
@@ -4797,7 +4797,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="88" spans="1:14">
+    <row r="88">
       <c r="A88" t="s">
         <v>100</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="89" spans="1:14">
+    <row r="89">
       <c r="A89" t="s">
         <v>101</v>
       </c>
@@ -4885,7 +4885,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="90" spans="1:14">
+    <row r="90">
       <c r="A90" t="s">
         <v>102</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="91" spans="1:14">
+    <row r="91">
       <c r="A91" t="s">
         <v>103</v>
       </c>
@@ -4973,7 +4973,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="92" spans="1:14">
+    <row r="92">
       <c r="A92" t="s">
         <v>104</v>
       </c>
@@ -5017,7 +5017,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="93" spans="1:14">
+    <row r="93">
       <c r="A93" t="s">
         <v>105</v>
       </c>
@@ -5061,7 +5061,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="94" spans="1:14">
+    <row r="94">
       <c r="A94" t="s">
         <v>106</v>
       </c>
@@ -5105,7 +5105,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="95" spans="1:14">
+    <row r="95">
       <c r="A95" t="s">
         <v>107</v>
       </c>
@@ -5149,7 +5149,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="96" spans="1:14">
+    <row r="96">
       <c r="A96" t="s">
         <v>108</v>
       </c>
@@ -5193,7 +5193,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="97" spans="1:14">
+    <row r="97">
       <c r="A97" t="s">
         <v>109</v>
       </c>
@@ -5237,7 +5237,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="98" spans="1:14">
+    <row r="98">
       <c r="A98" t="s">
         <v>110</v>
       </c>
@@ -5281,7 +5281,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="99" spans="1:14">
+    <row r="99">
       <c r="A99" t="s">
         <v>111</v>
       </c>
@@ -5325,7 +5325,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="100" spans="1:14">
+    <row r="100">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -5369,7 +5369,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="101" spans="1:14">
+    <row r="101">
       <c r="A101" t="s">
         <v>113</v>
       </c>

</xml_diff>